<commit_message>
defect-hub: update tracking for CleanCore_Defects_SAMPLE (3).xlsx (1/5 ticketed)
</commit_message>
<xml_diff>
--- a/tracking/2026-10-29/c47f3a51-aebe-47e7-8b8b-fc3a4b026a64_CleanCore_Defects_SAMPLE (3).xlsx
+++ b/tracking/2026-10-29/c47f3a51-aebe-47e7-8b8b-fc3a4b026a64_CleanCore_Defects_SAMPLE (3).xlsx
@@ -156,7 +156,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="89">
   <si>
     <t>Customer</t>
   </si>
@@ -245,31 +245,43 @@
     <t>mkarthik@smartshift.com</t>
   </si>
   <si>
+    <t>Approved</t>
+  </si>
+  <si>
+    <t>attachments/samples/st22_cast_dump.png|attachments/samples/analysis_cast_error.docx</t>
+  </si>
+  <si>
+    <t>JAIT-12</t>
+  </si>
+  <si>
+    <t>PROCESSED</t>
+  </si>
+  <si>
+    <t>2026-10-29T08:14:51.014Z</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>None</t>
+  </si>
+  <si>
+    <t>CDS view ZI_SalesDocItem returns duplicate rows after VBAP replacement</t>
+  </si>
+  <si>
+    <t>After replacing direct SELECT on VBAP with CDS view ZI_SalesDocItem the item count doubles for orders with multiple schedule lines (VBEP). Join cardinality on _ScheduleLine is MANY instead of ONE.</t>
+  </si>
+  <si>
+    <t>High</t>
+  </si>
+  <si>
     <t>In Progress</t>
   </si>
   <si>
-    <t>attachments/samples/st22_cast_dump.png|attachments/samples/analysis_cast_error.docx</t>
-  </si>
-  <si>
-    <t/>
+    <t>attachments/samples/cds_duplicate_rows.png|attachments/samples/cds_row_counts.xlsx</t>
   </si>
   <si>
     <t>PENDING</t>
-  </si>
-  <si>
-    <t>None</t>
-  </si>
-  <si>
-    <t>CDS view ZI_SalesDocItem returns duplicate rows after VBAP replacement</t>
-  </si>
-  <si>
-    <t>After replacing direct SELECT on VBAP with CDS view ZI_SalesDocItem the item count doubles for orders with multiple schedule lines (VBEP). Join cardinality on _ScheduleLine is MANY instead of ONE.</t>
-  </si>
-  <si>
-    <t>High</t>
-  </si>
-  <si>
-    <t>attachments/samples/cds_duplicate_rows.png|attachments/samples/cds_row_counts.xlsx</t>
   </si>
   <si>
     <t>P&amp;G</t>
@@ -948,16 +960,16 @@
         <v>32</v>
       </c>
       <c r="P2" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="Q2">
         <v>0</v>
       </c>
       <c r="R2" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="S2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="3" spans="1:19" x14ac:dyDescent="0.25">
@@ -974,10 +986,10 @@
         <v>22</v>
       </c>
       <c r="E3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="F3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="G3" t="s">
         <v>25</v>
@@ -986,7 +998,7 @@
         <v>26</v>
       </c>
       <c r="I3" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="J3" t="s">
         <v>28</v>
@@ -995,33 +1007,33 @@
         <v>28</v>
       </c>
       <c r="L3" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="M3" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="N3" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="O3" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="P3" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="Q3">
         <v>0</v>
       </c>
       <c r="R3" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="S3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="B4" t="s">
         <v>20</v>
@@ -1033,19 +1045,19 @@
         <v>22</v>
       </c>
       <c r="E4" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="F4" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="G4" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="H4" t="s">
         <v>26</v>
       </c>
       <c r="I4" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="J4" t="s">
         <v>28</v>
@@ -1054,33 +1066,33 @@
         <v>28</v>
       </c>
       <c r="L4" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="M4" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="N4" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="O4" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="P4" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="Q4">
         <v>0</v>
       </c>
       <c r="R4" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="S4" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="B5" t="s">
         <v>20</v>
@@ -1092,10 +1104,10 @@
         <v>22</v>
       </c>
       <c r="E5" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="F5" t="s">
-        <v>45</v>
+        <v>49</v>
       </c>
       <c r="G5" t="s">
         <v>25</v>
@@ -1104,7 +1116,7 @@
         <v>26</v>
       </c>
       <c r="I5" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="J5" t="s">
         <v>28</v>
@@ -1113,33 +1125,33 @@
         <v>28</v>
       </c>
       <c r="L5" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="M5" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="N5" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="O5" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="P5" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="Q5">
         <v>0</v>
       </c>
       <c r="R5" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="S5" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B6" t="s">
         <v>20</v>
@@ -1151,19 +1163,19 @@
         <v>22</v>
       </c>
       <c r="E6" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="F6" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="G6" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="H6" t="s">
         <v>26</v>
       </c>
       <c r="I6" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="J6" t="s">
         <v>28</v>
@@ -1172,28 +1184,28 @@
         <v>28</v>
       </c>
       <c r="L6" t="s">
-        <v>29</v>
+        <v>39</v>
       </c>
       <c r="M6" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="N6" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="O6" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="P6" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="Q6">
         <v>0</v>
       </c>
       <c r="R6" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="S6" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -1225,16 +1237,16 @@
         <v>4</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -1245,16 +1257,16 @@
         <v>23</v>
       </c>
       <c r="C2" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="D2" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="E2" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="F2" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -1265,196 +1277,196 @@
         <v>23</v>
       </c>
       <c r="C3" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="D3" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="E3" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="F3" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B4" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C4" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="D4" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="E4" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="F4" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B5" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="C5" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="D5" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="E5" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="F5" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B6" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C6" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="D6" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="E6" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="F6" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B7" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C7" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="D7" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="E7" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="F7" t="s">
-        <v>72</v>
+        <v>76</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B8" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C8" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="D8" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="E8" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="F8" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B9" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C9" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="D9" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="E9" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="F9" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B10" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="C10" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="D10" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="E10" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="F10" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B11" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C11" t="s">
-        <v>73</v>
+        <v>77</v>
       </c>
       <c r="D11" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="E11" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="F11" t="s">
-        <v>74</v>
+        <v>78</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="B12" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C12" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="D12" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="E12" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="F12" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -1488,35 +1500,35 @@
   <sheetData>
     <row r="1" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="B2" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C2" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="B3" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="C3" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
defect-hub: update tracking for CleanCore_Defects_SAMPLE (3).xlsx (2/5 ticketed)
</commit_message>
<xml_diff>
--- a/tracking/2026-10-29/c47f3a51-aebe-47e7-8b8b-fc3a4b026a64_CleanCore_Defects_SAMPLE (3).xlsx
+++ b/tracking/2026-10-29/c47f3a51-aebe-47e7-8b8b-fc3a4b026a64_CleanCore_Defects_SAMPLE (3).xlsx
@@ -156,7 +156,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="91">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="92">
   <si>
     <t>Customer</t>
   </si>
@@ -299,10 +299,13 @@
     <t>Medium</t>
   </si>
   <si>
-    <t>Changed Assignee</t>
-  </si>
-  <si>
     <t>attachments/samples/cfl_field_missing.png|attachments/samples/cfl_propagation_notes.docx|attachments/samples/mrp_type_comparison.xlsx</t>
+  </si>
+  <si>
+    <t>JAIT-13</t>
+  </si>
+  <si>
+    <t>2026-10-29T08:38:18.595Z</t>
   </si>
   <si>
     <t>knsspreddy@smartshift.com</t>
@@ -1072,28 +1075,28 @@
         <v>28</v>
       </c>
       <c r="L4" t="s">
+        <v>29</v>
+      </c>
+      <c r="M4" t="s">
         <v>47</v>
       </c>
-      <c r="M4" t="s">
+      <c r="N4" t="s">
         <v>48</v>
       </c>
-      <c r="N4" t="s">
-        <v>34</v>
-      </c>
       <c r="O4" t="s">
-        <v>41</v>
+        <v>32</v>
       </c>
       <c r="P4" t="s">
-        <v>34</v>
+        <v>49</v>
       </c>
       <c r="Q4">
         <v>0</v>
       </c>
       <c r="R4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="S4" t="s">
-        <v>39</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
@@ -1110,10 +1113,10 @@
         <v>22</v>
       </c>
       <c r="E5" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F5" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="G5" t="s">
         <v>25</v>
@@ -1122,7 +1125,7 @@
         <v>26</v>
       </c>
       <c r="I5" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="J5" t="s">
         <v>28</v>
@@ -1134,7 +1137,7 @@
         <v>39</v>
       </c>
       <c r="M5" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="N5" t="s">
         <v>34</v>
@@ -1157,7 +1160,7 @@
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B6" t="s">
         <v>20</v>
@@ -1169,13 +1172,13 @@
         <v>22</v>
       </c>
       <c r="E6" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H6" t="s">
         <v>26</v>
@@ -1193,7 +1196,7 @@
         <v>39</v>
       </c>
       <c r="M6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="N6" t="s">
         <v>34</v>
@@ -1243,16 +1246,16 @@
         <v>4</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -1263,16 +1266,16 @@
         <v>23</v>
       </c>
       <c r="C2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -1283,16 +1286,16 @@
         <v>23</v>
       </c>
       <c r="C3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F3" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -1303,16 +1306,16 @@
         <v>36</v>
       </c>
       <c r="C4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -1323,76 +1326,76 @@
         <v>36</v>
       </c>
       <c r="C5" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="D5" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F5" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="B6" t="s">
         <v>43</v>
       </c>
       <c r="C6" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F6" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="B7" t="s">
         <v>43</v>
       </c>
       <c r="C7" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="D7" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E7" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F7" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="B8" t="s">
         <v>43</v>
       </c>
       <c r="C8" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D8" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E8" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F8" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -1400,19 +1403,19 @@
         <v>34</v>
       </c>
       <c r="B9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C9" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="D9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E9" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F9" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -1420,19 +1423,19 @@
         <v>34</v>
       </c>
       <c r="B10" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C10" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="D10" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E10" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F10" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -1440,19 +1443,19 @@
         <v>34</v>
       </c>
       <c r="B11" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C11" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="D11" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F11" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -1460,19 +1463,19 @@
         <v>34</v>
       </c>
       <c r="B12" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C12" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="D12" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E12" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="F12" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
   </sheetData>
@@ -1506,35 +1509,35 @@
   <sheetData>
     <row r="1" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B2" t="s">
         <v>34</v>
       </c>
       <c r="C2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="B3" t="s">
         <v>34</v>
       </c>
       <c r="C3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
defect-hub: update tracking for CleanCore_Defects_SAMPLE (3).xlsx (3/5 ticketed)
</commit_message>
<xml_diff>
--- a/tracking/2026-10-29/c47f3a51-aebe-47e7-8b8b-fc3a4b026a64_CleanCore_Defects_SAMPLE (3).xlsx
+++ b/tracking/2026-10-29/c47f3a51-aebe-47e7-8b8b-fc3a4b026a64_CleanCore_Defects_SAMPLE (3).xlsx
@@ -156,7 +156,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="95">
   <si>
     <t>Customer</t>
   </si>
@@ -275,58 +275,61 @@
     <t>High</t>
   </si>
   <si>
-    <t>Changed Assignee</t>
-  </si>
-  <si>
     <t>attachments/samples/cds_duplicate_rows.png|attachments/samples/cds_row_counts.xlsx</t>
   </si>
   <si>
+    <t>JAIT-16</t>
+  </si>
+  <si>
+    <t>2026-10-30T07:10:18.608Z</t>
+  </si>
+  <si>
+    <t>asarath@smartshift.com</t>
+  </si>
+  <si>
+    <t>P&amp;G</t>
+  </si>
+  <si>
+    <t>CFL: custom field ZZ_BATCH_ORIGIN not propagated from goods receipt to MATDOC</t>
+  </si>
+  <si>
+    <t>Field created in Custom Fields app for Material Document Item. Value is entered via Post Goods Receipt but MATDOC.ZZ_BATCH_ORIGIN stays initial. Check propagation for the business context.</t>
+  </si>
+  <si>
+    <t>Task</t>
+  </si>
+  <si>
+    <t>Medium</t>
+  </si>
+  <si>
+    <t>attachments/samples/cfl_field_missing.png|attachments/samples/cfl_propagation_notes.docx|attachments/samples/mrp_type_comparison.xlsx</t>
+  </si>
+  <si>
+    <t>JAIT-13</t>
+  </si>
+  <si>
+    <t>2026-10-29T08:38:18.595Z</t>
+  </si>
+  <si>
+    <t>knsspreddy@smartshift.com</t>
+  </si>
+  <si>
+    <t>AMF syntax failure: missing period after DEFINE ROLE in ZAMF_AUTH_SALES</t>
+  </si>
+  <si>
+    <t>Activation fails: 'The statement DEFINE ROLE must end with a period' at line 17 of ZAMF_AUTH_SALES. Introduced by the automated formatter in ADT.</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>In Progress</t>
+  </si>
+  <si>
+    <t>attachments/samples/st22_cast_dump.png|https://docs.github.com/en/rest/repos/contents</t>
+  </si>
+  <si>
     <t>PENDING</t>
-  </si>
-  <si>
-    <t>asarath@smartshift.com</t>
-  </si>
-  <si>
-    <t>In Progress</t>
-  </si>
-  <si>
-    <t>P&amp;G</t>
-  </si>
-  <si>
-    <t>CFL: custom field ZZ_BATCH_ORIGIN not propagated from goods receipt to MATDOC</t>
-  </si>
-  <si>
-    <t>Field created in Custom Fields app for Material Document Item. Value is entered via Post Goods Receipt but MATDOC.ZZ_BATCH_ORIGIN stays initial. Check propagation for the business context.</t>
-  </si>
-  <si>
-    <t>Task</t>
-  </si>
-  <si>
-    <t>Medium</t>
-  </si>
-  <si>
-    <t>attachments/samples/cfl_field_missing.png|attachments/samples/cfl_propagation_notes.docx|attachments/samples/mrp_type_comparison.xlsx</t>
-  </si>
-  <si>
-    <t>JAIT-13</t>
-  </si>
-  <si>
-    <t>2026-10-29T08:38:18.595Z</t>
-  </si>
-  <si>
-    <t>knsspreddy@smartshift.com</t>
-  </si>
-  <si>
-    <t>AMF syntax failure: missing period after DEFINE ROLE in ZAMF_AUTH_SALES</t>
-  </si>
-  <si>
-    <t>Activation fails: 'The statement DEFINE ROLE must end with a period' at line 17 of ZAMF_AUTH_SALES. Introduced by the automated formatter in ADT.</t>
-  </si>
-  <si>
-    <t>Low</t>
-  </si>
-  <si>
-    <t>attachments/samples/st22_cast_dump.png|https://docs.github.com/en/rest/repos/contents</t>
   </si>
   <si>
     <t>VOITH</t>
@@ -1022,19 +1025,19 @@
         <v>28</v>
       </c>
       <c r="L3" t="s">
+        <v>29</v>
+      </c>
+      <c r="M3" t="s">
         <v>39</v>
       </c>
-      <c r="M3" t="s">
+      <c r="N3" t="s">
         <v>40</v>
       </c>
-      <c r="N3" t="s">
-        <v>34</v>
-      </c>
       <c r="O3" t="s">
+        <v>32</v>
+      </c>
+      <c r="P3" t="s">
         <v>41</v>
-      </c>
-      <c r="P3" t="s">
-        <v>34</v>
       </c>
       <c r="Q3">
         <v>2</v>
@@ -1043,12 +1046,12 @@
         <v>42</v>
       </c>
       <c r="S3" t="s">
-        <v>43</v>
+        <v>29</v>
       </c>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B4" t="s">
         <v>20</v>
@@ -1060,19 +1063,19 @@
         <v>22</v>
       </c>
       <c r="E4" t="s">
+        <v>44</v>
+      </c>
+      <c r="F4" t="s">
         <v>45</v>
       </c>
-      <c r="F4" t="s">
+      <c r="G4" t="s">
         <v>46</v>
-      </c>
-      <c r="G4" t="s">
-        <v>47</v>
       </c>
       <c r="H4" t="s">
         <v>26</v>
       </c>
       <c r="I4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J4" t="s">
         <v>28</v>
@@ -1084,22 +1087,22 @@
         <v>29</v>
       </c>
       <c r="M4" t="s">
+        <v>48</v>
+      </c>
+      <c r="N4" t="s">
         <v>49</v>
-      </c>
-      <c r="N4" t="s">
-        <v>50</v>
       </c>
       <c r="O4" t="s">
         <v>32</v>
       </c>
       <c r="P4" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="Q4">
         <v>2</v>
       </c>
       <c r="R4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="S4" t="s">
         <v>29</v>
@@ -1107,7 +1110,7 @@
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B5" t="s">
         <v>20</v>
@@ -1119,10 +1122,10 @@
         <v>22</v>
       </c>
       <c r="E5" t="s">
+        <v>52</v>
+      </c>
+      <c r="F5" t="s">
         <v>53</v>
-      </c>
-      <c r="F5" t="s">
-        <v>54</v>
       </c>
       <c r="G5" t="s">
         <v>25</v>
@@ -1131,7 +1134,7 @@
         <v>26</v>
       </c>
       <c r="I5" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="J5" t="s">
         <v>28</v>
@@ -1140,7 +1143,7 @@
         <v>28</v>
       </c>
       <c r="L5" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="M5" t="s">
         <v>56</v>
@@ -1149,7 +1152,7 @@
         <v>34</v>
       </c>
       <c r="O5" t="s">
-        <v>41</v>
+        <v>57</v>
       </c>
       <c r="P5" t="s">
         <v>34</v>
@@ -1166,7 +1169,7 @@
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B6" t="s">
         <v>20</v>
@@ -1178,19 +1181,19 @@
         <v>22</v>
       </c>
       <c r="E6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="F6" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="G6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="H6" t="s">
         <v>26</v>
       </c>
       <c r="I6" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="J6" t="s">
         <v>28</v>
@@ -1199,16 +1202,16 @@
         <v>28</v>
       </c>
       <c r="L6" t="s">
-        <v>43</v>
+        <v>55</v>
       </c>
       <c r="M6" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="N6" t="s">
         <v>34</v>
       </c>
       <c r="O6" t="s">
-        <v>41</v>
+        <v>57</v>
       </c>
       <c r="P6" t="s">
         <v>34</v>
@@ -1252,16 +1255,16 @@
         <v>4</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -1272,16 +1275,16 @@
         <v>23</v>
       </c>
       <c r="C2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E2" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F2" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -1292,116 +1295,116 @@
         <v>23</v>
       </c>
       <c r="C3" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D3" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F3" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B4" t="s">
         <v>36</v>
       </c>
       <c r="C4" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="D4" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E4" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F4" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>34</v>
+        <v>40</v>
       </c>
       <c r="B5" t="s">
         <v>36</v>
       </c>
       <c r="C5" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="D5" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E5" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F5" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B6" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C6" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="D6" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E6" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F6" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B7" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C7" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D7" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E7" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F7" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B8" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C8" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D8" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E8" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F8" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -1409,19 +1412,19 @@
         <v>34</v>
       </c>
       <c r="B9" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C9" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="D9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E9" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F9" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -1429,19 +1432,19 @@
         <v>34</v>
       </c>
       <c r="B10" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C10" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="D10" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E10" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F10" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -1449,19 +1452,19 @@
         <v>34</v>
       </c>
       <c r="B11" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C11" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D11" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="E11" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F11" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -1469,19 +1472,19 @@
         <v>34</v>
       </c>
       <c r="B12" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="C12" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="D12" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E12" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="F12" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -1515,35 +1518,35 @@
   <sheetData>
     <row r="1" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B2" t="s">
         <v>34</v>
       </c>
       <c r="C2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B3" t="s">
         <v>34</v>
       </c>
       <c r="C3" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
defect-hub: update tracking for CleanCore_Defects_SAMPLE (3).xlsx (4/5 ticketed)
</commit_message>
<xml_diff>
--- a/tracking/2026-10-29/c47f3a51-aebe-47e7-8b8b-fc3a4b026a64_CleanCore_Defects_SAMPLE (3).xlsx
+++ b/tracking/2026-10-29/c47f3a51-aebe-47e7-8b8b-fc3a4b026a64_CleanCore_Defects_SAMPLE (3).xlsx
@@ -156,7 +156,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="97">
   <si>
     <t>Customer</t>
   </si>
@@ -323,28 +323,34 @@
     <t>Low</t>
   </si>
   <si>
+    <t>attachments/samples/st22_cast_dump.png|https://docs.github.com/en/rest/repos/contents</t>
+  </si>
+  <si>
+    <t>JAIT-17</t>
+  </si>
+  <si>
+    <t>2026-10-30T07:45:05.433Z</t>
+  </si>
+  <si>
+    <t>VOITH</t>
+  </si>
+  <si>
+    <t>Table-to-CDS: MARA/MARC join replaced by I_Product loses plant-specific MRP type</t>
+  </si>
+  <si>
+    <t>ZMM_MRP_OVERVIEW previously joined MARA and MARC. After moving to CDS I_Product with association _ProductPlant the MRP type (DISMM) is blank for plants 1010 and 1020.</t>
+  </si>
+  <si>
+    <t>Story</t>
+  </si>
+  <si>
     <t>In Progress</t>
   </si>
   <si>
-    <t>attachments/samples/st22_cast_dump.png|https://docs.github.com/en/rest/repos/contents</t>
+    <t>attachments/samples/mrp_type_comparison.xlsx|attachments/samples/analysis_cast_error.docx</t>
   </si>
   <si>
     <t>PENDING</t>
-  </si>
-  <si>
-    <t>VOITH</t>
-  </si>
-  <si>
-    <t>Table-to-CDS: MARA/MARC join replaced by I_Product loses plant-specific MRP type</t>
-  </si>
-  <si>
-    <t>ZMM_MRP_OVERVIEW previously joined MARA and MARC. After moving to CDS I_Product with association _ProductPlant the MRP type (DISMM) is blank for plants 1010 and 1020.</t>
-  </si>
-  <si>
-    <t>Story</t>
-  </si>
-  <si>
-    <t>attachments/samples/mrp_type_comparison.xlsx|attachments/samples/analysis_cast_error.docx</t>
   </si>
   <si>
     <t>File / link</t>
@@ -1143,19 +1149,19 @@
         <v>28</v>
       </c>
       <c r="L5" t="s">
+        <v>29</v>
+      </c>
+      <c r="M5" t="s">
         <v>55</v>
       </c>
-      <c r="M5" t="s">
+      <c r="N5" t="s">
         <v>56</v>
       </c>
-      <c r="N5" t="s">
-        <v>34</v>
-      </c>
       <c r="O5" t="s">
+        <v>32</v>
+      </c>
+      <c r="P5" t="s">
         <v>57</v>
-      </c>
-      <c r="P5" t="s">
-        <v>34</v>
       </c>
       <c r="Q5">
         <v>2</v>
@@ -1202,16 +1208,16 @@
         <v>28</v>
       </c>
       <c r="L6" t="s">
-        <v>55</v>
+        <v>62</v>
       </c>
       <c r="M6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="N6" t="s">
         <v>34</v>
       </c>
       <c r="O6" t="s">
-        <v>57</v>
+        <v>64</v>
       </c>
       <c r="P6" t="s">
         <v>34</v>
@@ -1255,16 +1261,16 @@
         <v>4</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -1275,16 +1281,16 @@
         <v>23</v>
       </c>
       <c r="C2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D2" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -1295,16 +1301,16 @@
         <v>23</v>
       </c>
       <c r="C3" t="s">
+        <v>73</v>
+      </c>
+      <c r="D3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E3" t="s">
         <v>71</v>
       </c>
-      <c r="D3" t="s">
-        <v>72</v>
-      </c>
-      <c r="E3" t="s">
-        <v>69</v>
-      </c>
       <c r="F3" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -1315,16 +1321,16 @@
         <v>36</v>
       </c>
       <c r="C4" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="D4" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E4" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F4" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -1335,16 +1341,16 @@
         <v>36</v>
       </c>
       <c r="C5" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D5" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="E5" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F5" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -1355,16 +1361,16 @@
         <v>44</v>
       </c>
       <c r="C6" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D6" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E6" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F6" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -1375,16 +1381,16 @@
         <v>44</v>
       </c>
       <c r="C7" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D7" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="E7" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F7" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -1395,56 +1401,56 @@
         <v>44</v>
       </c>
       <c r="C8" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D8" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="E8" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F8" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>34</v>
+        <v>56</v>
       </c>
       <c r="B9" t="s">
         <v>52</v>
       </c>
       <c r="C9" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D9" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="E9" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F9" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>34</v>
+        <v>56</v>
       </c>
       <c r="B10" t="s">
         <v>52</v>
       </c>
       <c r="C10" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="D10" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="E10" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F10" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
@@ -1455,16 +1461,16 @@
         <v>59</v>
       </c>
       <c r="C11" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="D11" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="E11" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F11" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
@@ -1475,16 +1481,16 @@
         <v>59</v>
       </c>
       <c r="C12" t="s">
+        <v>73</v>
+      </c>
+      <c r="D12" t="s">
+        <v>74</v>
+      </c>
+      <c r="E12" t="s">
         <v>71</v>
       </c>
-      <c r="D12" t="s">
-        <v>72</v>
-      </c>
-      <c r="E12" t="s">
-        <v>69</v>
-      </c>
       <c r="F12" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -1518,35 +1524,35 @@
   <sheetData>
     <row r="1" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="B1" s="4" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="B2" t="s">
         <v>34</v>
       </c>
       <c r="C2" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="B3" t="s">
         <v>34</v>
       </c>
       <c r="C3" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
defect-hub: update tracking for CleanCore_Defects_SAMPLE (3).xlsx (5/5 ticketed)
</commit_message>
<xml_diff>
--- a/tracking/2026-10-29/c47f3a51-aebe-47e7-8b8b-fc3a4b026a64_CleanCore_Defects_SAMPLE (3).xlsx
+++ b/tracking/2026-10-29/c47f3a51-aebe-47e7-8b8b-fc3a4b026a64_CleanCore_Defects_SAMPLE (3).xlsx
@@ -156,7 +156,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="190" uniqueCount="98">
   <si>
     <t>Customer</t>
   </si>
@@ -344,19 +344,16 @@
     <t>Story</t>
   </si>
   <si>
-    <t>Changed Assignee</t>
-  </si>
-  <si>
     <t>attachments/samples/mrp_type_comparison.xlsx|attachments/samples/analysis_cast_error.docx</t>
   </si>
   <si>
-    <t>PENDING</t>
+    <t>JAIT-18</t>
+  </si>
+  <si>
+    <t>2026-10-30T07:51:07.372Z</t>
   </si>
   <si>
     <t>rcbabu@smartshift.com</t>
-  </si>
-  <si>
-    <t>In Progress</t>
   </si>
   <si>
     <t>File / link</t>
@@ -1214,19 +1211,19 @@
         <v>28</v>
       </c>
       <c r="L6" t="s">
+        <v>29</v>
+      </c>
+      <c r="M6" t="s">
         <v>62</v>
       </c>
-      <c r="M6" t="s">
+      <c r="N6" t="s">
         <v>63</v>
       </c>
-      <c r="N6" t="s">
-        <v>34</v>
-      </c>
       <c r="O6" t="s">
+        <v>32</v>
+      </c>
+      <c r="P6" t="s">
         <v>64</v>
-      </c>
-      <c r="P6" t="s">
-        <v>34</v>
       </c>
       <c r="Q6">
         <v>2</v>
@@ -1235,7 +1232,7 @@
         <v>65</v>
       </c>
       <c r="S6" t="s">
-        <v>66</v>
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -1267,16 +1264,16 @@
         <v>4</v>
       </c>
       <c r="C1" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="D1" s="4" t="s">
         <v>67</v>
       </c>
-      <c r="D1" s="4" t="s">
+      <c r="E1" s="4" t="s">
         <v>68</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>69</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.25">
@@ -1287,16 +1284,16 @@
         <v>23</v>
       </c>
       <c r="C2" t="s">
+        <v>70</v>
+      </c>
+      <c r="D2" t="s">
         <v>71</v>
       </c>
-      <c r="D2" t="s">
+      <c r="E2" t="s">
         <v>72</v>
       </c>
-      <c r="E2" t="s">
+      <c r="F2" t="s">
         <v>73</v>
-      </c>
-      <c r="F2" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="3" spans="1:6" x14ac:dyDescent="0.25">
@@ -1307,16 +1304,16 @@
         <v>23</v>
       </c>
       <c r="C3" t="s">
+        <v>74</v>
+      </c>
+      <c r="D3" t="s">
         <v>75</v>
       </c>
-      <c r="D3" t="s">
+      <c r="E3" t="s">
+        <v>72</v>
+      </c>
+      <c r="F3" t="s">
         <v>76</v>
-      </c>
-      <c r="E3" t="s">
-        <v>73</v>
-      </c>
-      <c r="F3" t="s">
-        <v>77</v>
       </c>
     </row>
     <row r="4" spans="1:6" x14ac:dyDescent="0.25">
@@ -1327,16 +1324,16 @@
         <v>36</v>
       </c>
       <c r="C4" t="s">
+        <v>77</v>
+      </c>
+      <c r="D4" t="s">
+        <v>71</v>
+      </c>
+      <c r="E4" t="s">
+        <v>72</v>
+      </c>
+      <c r="F4" t="s">
         <v>78</v>
-      </c>
-      <c r="D4" t="s">
-        <v>72</v>
-      </c>
-      <c r="E4" t="s">
-        <v>73</v>
-      </c>
-      <c r="F4" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.25">
@@ -1347,16 +1344,16 @@
         <v>36</v>
       </c>
       <c r="C5" t="s">
+        <v>79</v>
+      </c>
+      <c r="D5" t="s">
         <v>80</v>
       </c>
-      <c r="D5" t="s">
+      <c r="E5" t="s">
+        <v>72</v>
+      </c>
+      <c r="F5" t="s">
         <v>81</v>
-      </c>
-      <c r="E5" t="s">
-        <v>73</v>
-      </c>
-      <c r="F5" t="s">
-        <v>82</v>
       </c>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.25">
@@ -1367,16 +1364,16 @@
         <v>44</v>
       </c>
       <c r="C6" t="s">
+        <v>82</v>
+      </c>
+      <c r="D6" t="s">
+        <v>71</v>
+      </c>
+      <c r="E6" t="s">
+        <v>72</v>
+      </c>
+      <c r="F6" t="s">
         <v>83</v>
-      </c>
-      <c r="D6" t="s">
-        <v>72</v>
-      </c>
-      <c r="E6" t="s">
-        <v>73</v>
-      </c>
-      <c r="F6" t="s">
-        <v>84</v>
       </c>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.25">
@@ -1387,16 +1384,16 @@
         <v>44</v>
       </c>
       <c r="C7" t="s">
+        <v>84</v>
+      </c>
+      <c r="D7" t="s">
+        <v>75</v>
+      </c>
+      <c r="E7" t="s">
+        <v>72</v>
+      </c>
+      <c r="F7" t="s">
         <v>85</v>
-      </c>
-      <c r="D7" t="s">
-        <v>76</v>
-      </c>
-      <c r="E7" t="s">
-        <v>73</v>
-      </c>
-      <c r="F7" t="s">
-        <v>86</v>
       </c>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.25">
@@ -1407,16 +1404,16 @@
         <v>44</v>
       </c>
       <c r="C8" t="s">
+        <v>86</v>
+      </c>
+      <c r="D8" t="s">
+        <v>80</v>
+      </c>
+      <c r="E8" t="s">
+        <v>72</v>
+      </c>
+      <c r="F8" t="s">
         <v>87</v>
-      </c>
-      <c r="D8" t="s">
-        <v>81</v>
-      </c>
-      <c r="E8" t="s">
-        <v>73</v>
-      </c>
-      <c r="F8" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.25">
@@ -1427,16 +1424,16 @@
         <v>52</v>
       </c>
       <c r="C9" t="s">
+        <v>70</v>
+      </c>
+      <c r="D9" t="s">
         <v>71</v>
       </c>
-      <c r="D9" t="s">
+      <c r="E9" t="s">
         <v>72</v>
       </c>
-      <c r="E9" t="s">
+      <c r="F9" t="s">
         <v>73</v>
-      </c>
-      <c r="F9" t="s">
-        <v>74</v>
       </c>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.25">
@@ -1447,56 +1444,56 @@
         <v>52</v>
       </c>
       <c r="C10" t="s">
+        <v>88</v>
+      </c>
+      <c r="D10" t="s">
         <v>89</v>
       </c>
-      <c r="D10" t="s">
+      <c r="E10" t="s">
+        <v>72</v>
+      </c>
+      <c r="F10" t="s">
         <v>90</v>
-      </c>
-      <c r="E10" t="s">
-        <v>73</v>
-      </c>
-      <c r="F10" t="s">
-        <v>91</v>
       </c>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>34</v>
+        <v>63</v>
       </c>
       <c r="B11" t="s">
         <v>59</v>
       </c>
       <c r="C11" t="s">
+        <v>86</v>
+      </c>
+      <c r="D11" t="s">
+        <v>80</v>
+      </c>
+      <c r="E11" t="s">
+        <v>72</v>
+      </c>
+      <c r="F11" t="s">
         <v>87</v>
-      </c>
-      <c r="D11" t="s">
-        <v>81</v>
-      </c>
-      <c r="E11" t="s">
-        <v>73</v>
-      </c>
-      <c r="F11" t="s">
-        <v>88</v>
       </c>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>34</v>
+        <v>63</v>
       </c>
       <c r="B12" t="s">
         <v>59</v>
       </c>
       <c r="C12" t="s">
+        <v>74</v>
+      </c>
+      <c r="D12" t="s">
         <v>75</v>
       </c>
-      <c r="D12" t="s">
+      <c r="E12" t="s">
+        <v>72</v>
+      </c>
+      <c r="F12" t="s">
         <v>76</v>
-      </c>
-      <c r="E12" t="s">
-        <v>73</v>
-      </c>
-      <c r="F12" t="s">
-        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -1530,35 +1527,35 @@
   <sheetData>
     <row r="1" spans="1:3" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
+        <v>91</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>92</v>
       </c>
-      <c r="B1" s="4" t="s">
+      <c r="C1" s="4" t="s">
         <v>93</v>
-      </c>
-      <c r="C1" s="4" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="B2" t="s">
         <v>34</v>
       </c>
       <c r="C2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="B3" t="s">
         <v>34</v>
       </c>
       <c r="C3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
   </sheetData>

</xml_diff>